<commit_message>
Incorporate new clean data and separate different approaches
</commit_message>
<xml_diff>
--- a/R Markdown analysis/division_drug_search_proptest_results.xlsx
+++ b/R Markdown analysis/division_drug_search_proptest_results.xlsx
@@ -424,7 +424,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NWMR Division 3</t>
+          <t>NWMR Division 3 (Brimbank, Melton)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NWMR Division 2</t>
+          <t>NWMR Division 2 (Hobsons Bay, Maribyrnong, Wyndham)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -518,7 +518,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NWMR Division 4</t>
+          <t>NWMR Division 4 (Hume, Moonee Valley, Merri-bek)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Eastern Region Division 1</t>
+          <t>Eastern Region Division 1 (Boroondara, Manningham, Monash, Whitehorse)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SMR Division 4</t>
+          <t>SMR Division 4 (Frankston, Mornington)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NWMR Division 5</t>
+          <t>NWMR Division 5 (Banyule, Darebin, Nillumbik, Whittlesea)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -706,7 +706,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Eastern Region Division 2</t>
+          <t>Eastern Region Division 2 (Knox, Maroondah, Yarra Ranges)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NWMR Division 1</t>
+          <t>NWMR Division 1 (Melbourne, Yarra)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -800,7 +800,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SMR Division 2</t>
+          <t>SMR Division 2 (Glen Eira, Kingston)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -847,7 +847,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SMR Division 3</t>
+          <t>SMR Division 3 (Cardinia, Casey, Dandenong)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SMR Division 1</t>
+          <t>SMR Division 1 (Port Phillip, Stonnington)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">

</xml_diff>